<commit_message>
Profil Tren Agen: filter strictly real SCO only, remove cabang filter
</commit_message>
<xml_diff>
--- a/KPI_SCO.xlsx
+++ b/KPI_SCO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WEB REPORT\pages\sco\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C78F4D8C-41C8-463B-8F44-E7A590338944}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{640210A1-815D-480C-A8ED-CB8CED1E1288}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -451,6 +451,76 @@
     <xf numFmtId="167" fontId="9" fillId="0" borderId="2" xfId="3" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="11" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="11" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="9" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="17" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -484,78 +554,8 @@
     <xf numFmtId="0" fontId="10" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="9" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="11" fillId="0" borderId="2" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="11" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="9" fillId="0" borderId="2" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="17" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -564,27 +564,7 @@
     <cellStyle name="Normal 2" xfId="3" xr:uid="{DBE81324-0B33-4294-821C-0B109FBA027A}"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF9C0006"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFFC7CE"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <font>
         <color rgb="FF9C0006"/>
@@ -30859,7 +30839,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B432E2F1-95BC-47FA-AE10-C07324981276}">
-  <dimension ref="A1:Q14"/>
+  <dimension ref="A1:Q15"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.85546875" bestFit="1" customWidth="1"/>
@@ -30868,7 +30848,7 @@
     <col min="4" max="4" width="6.5703125" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="5.85546875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="6.42578125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="6.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="8.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="7.5703125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="6.5703125" bestFit="1" customWidth="1"/>
@@ -30880,780 +30860,818 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="36" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="13">
+      <c r="B1" s="37">
         <v>0.3</v>
       </c>
-      <c r="C1" s="14"/>
-      <c r="D1" s="15"/>
-      <c r="E1" s="16">
+      <c r="C1" s="38"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="40">
         <v>0.2</v>
       </c>
-      <c r="F1" s="17"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="19">
+      <c r="F1" s="41"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="43">
         <v>0.3</v>
       </c>
-      <c r="I1" s="20"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="19">
+      <c r="I1" s="44"/>
+      <c r="J1" s="45"/>
+      <c r="K1" s="43">
         <v>0.2</v>
       </c>
-      <c r="L1" s="20"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="22" t="s">
+      <c r="L1" s="44"/>
+      <c r="M1" s="45"/>
+      <c r="N1" s="46" t="s">
         <v>24</v>
       </c>
-      <c r="O1" s="23"/>
-      <c r="P1" s="24" t="s">
+      <c r="O1" s="12"/>
+      <c r="P1" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="Q1" s="25" t="s">
+      <c r="Q1" s="26" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="12"/>
-      <c r="B2" s="26" t="s">
+      <c r="A2" s="36"/>
+      <c r="B2" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="27"/>
-      <c r="D2" s="28"/>
-      <c r="E2" s="29" t="s">
+      <c r="C2" s="28"/>
+      <c r="D2" s="29"/>
+      <c r="E2" s="30" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="30"/>
-      <c r="G2" s="31"/>
-      <c r="H2" s="32" t="s">
+      <c r="F2" s="31"/>
+      <c r="G2" s="32"/>
+      <c r="H2" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="I2" s="33"/>
-      <c r="J2" s="34"/>
-      <c r="K2" s="32" t="s">
+      <c r="I2" s="34"/>
+      <c r="J2" s="35"/>
+      <c r="K2" s="33" t="s">
         <v>30</v>
       </c>
-      <c r="L2" s="33"/>
-      <c r="M2" s="34"/>
-      <c r="N2" s="35"/>
-      <c r="O2" s="23"/>
-      <c r="P2" s="36"/>
-      <c r="Q2" s="25"/>
+      <c r="L2" s="34"/>
+      <c r="M2" s="35"/>
+      <c r="N2" s="47"/>
+      <c r="O2" s="12"/>
+      <c r="P2" s="24"/>
+      <c r="Q2" s="26"/>
     </row>
     <row r="3" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="12"/>
-      <c r="B3" s="37" t="s">
+      <c r="A3" s="36"/>
+      <c r="B3" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="C3" s="37" t="s">
+      <c r="C3" s="13" t="s">
         <v>32</v>
       </c>
-      <c r="D3" s="37" t="s">
+      <c r="D3" s="13" t="s">
         <v>33</v>
       </c>
-      <c r="E3" s="38" t="s">
+      <c r="E3" s="14" t="s">
         <v>31</v>
       </c>
-      <c r="F3" s="38" t="s">
+      <c r="F3" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="G3" s="38" t="s">
+      <c r="G3" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="H3" s="39" t="s">
+      <c r="H3" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="I3" s="39" t="s">
+      <c r="I3" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="J3" s="39" t="s">
+      <c r="J3" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="K3" s="39" t="s">
+      <c r="K3" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="L3" s="39" t="s">
+      <c r="L3" s="15" t="s">
         <v>32</v>
       </c>
-      <c r="M3" s="39" t="s">
+      <c r="M3" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="N3" s="35"/>
-      <c r="O3" s="23"/>
-      <c r="P3" s="40"/>
-      <c r="Q3" s="25"/>
+      <c r="N3" s="47"/>
+      <c r="O3" s="12"/>
+      <c r="P3" s="25"/>
+      <c r="Q3" s="26"/>
     </row>
     <row r="4" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A4" s="41">
+      <c r="A4" s="16">
         <v>45962</v>
       </c>
-      <c r="B4" s="42">
+      <c r="B4" s="17">
         <f>60</f>
         <v>60</v>
       </c>
-      <c r="C4" s="42">
+      <c r="C4" s="17">
         <v>8</v>
       </c>
-      <c r="D4" s="43">
+      <c r="D4" s="18">
         <f>C4/B4</f>
         <v>0.13333333333333333</v>
       </c>
-      <c r="E4" s="42">
+      <c r="E4" s="17">
         <f>150</f>
         <v>150</v>
       </c>
       <c r="F4" s="11">
         <v>11.9</v>
       </c>
-      <c r="G4" s="43">
+      <c r="G4" s="18">
         <f t="shared" ref="G4:G12" si="0">IFERROR(F4/E4,0)</f>
         <v>7.9333333333333339E-2</v>
       </c>
-      <c r="H4" s="42">
+      <c r="H4" s="17">
         <f>20000</f>
         <v>20000</v>
       </c>
-      <c r="I4" s="42">
+      <c r="I4" s="17">
         <v>1934</v>
       </c>
-      <c r="J4" s="43">
+      <c r="J4" s="18">
         <f t="shared" ref="J4:J12" si="1">IFERROR(I4/H4,0)</f>
         <v>9.6699999999999994E-2</v>
       </c>
-      <c r="K4" s="42">
+      <c r="K4" s="17">
         <f>200</f>
         <v>200</v>
       </c>
-      <c r="L4" s="42">
+      <c r="L4" s="17">
         <v>418</v>
       </c>
-      <c r="M4" s="43">
+      <c r="M4" s="18">
         <f t="shared" ref="M4:M12" si="2">IFERROR(L4/K4,0)</f>
         <v>2.09</v>
       </c>
-      <c r="N4" s="43">
+      <c r="N4" s="18">
         <f>(D4*$B$1)+(G4*$E$1)+(J4*$H$1)+(M4*$K$1)</f>
         <v>0.50287666666666664</v>
       </c>
-      <c r="O4" s="44"/>
-      <c r="P4" s="45">
+      <c r="O4" s="19"/>
+      <c r="P4" s="20">
         <f>IF($O4&gt;120%,120%,IF($O4&gt;=70%,N4,IF($O4&gt;=60%,50%,0%)))</f>
         <v>0</v>
       </c>
-      <c r="Q4" s="46">
+      <c r="Q4" s="21">
         <f>((F4*31)+(I4+L4))*50*P4</f>
         <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A5" s="47">
+      <c r="A5" s="22">
         <v>45992</v>
       </c>
-      <c r="B5" s="42">
+      <c r="B5" s="17">
         <f>60</f>
         <v>60</v>
       </c>
-      <c r="C5" s="42">
+      <c r="C5" s="17">
         <v>0</v>
       </c>
-      <c r="D5" s="43">
+      <c r="D5" s="18">
         <f t="shared" ref="D5:D12" si="3">C5/B5</f>
         <v>0</v>
       </c>
-      <c r="E5" s="42">
+      <c r="E5" s="17">
         <f>150</f>
         <v>150</v>
       </c>
       <c r="F5" s="11">
         <v>0</v>
       </c>
-      <c r="G5" s="43">
+      <c r="G5" s="18">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H5" s="42">
+      <c r="H5" s="17">
         <f>20000</f>
         <v>20000</v>
       </c>
-      <c r="I5" s="42">
+      <c r="I5" s="17">
         <v>2247</v>
       </c>
-      <c r="J5" s="43">
+      <c r="J5" s="18">
         <f t="shared" si="1"/>
         <v>0.11235000000000001</v>
       </c>
-      <c r="K5" s="42">
+      <c r="K5" s="17">
         <f>200</f>
         <v>200</v>
       </c>
-      <c r="L5" s="42">
+      <c r="L5" s="17">
         <v>326</v>
       </c>
-      <c r="M5" s="43">
+      <c r="M5" s="18">
         <f t="shared" si="2"/>
         <v>1.63</v>
       </c>
-      <c r="N5" s="43">
+      <c r="N5" s="18">
         <f t="shared" ref="N5:N12" si="4">(D5*$B$1)+(G5*$E$1)+(J5*$H$1)+(M5*$K$1)</f>
         <v>0.359705</v>
       </c>
-      <c r="O5" s="23"/>
-      <c r="P5" s="45">
+      <c r="O5" s="12"/>
+      <c r="P5" s="20">
         <f t="shared" ref="P5:P12" si="5">IF($O5&gt;120%,120%,IF($O5&gt;=70%,N5,IF($O5&gt;=60%,50%,0%)))</f>
         <v>0</v>
       </c>
-      <c r="Q5" s="46">
+      <c r="Q5" s="21">
         <f t="shared" ref="Q5:Q12" si="6">((F5*31)+(I5+L5))*50*P5</f>
         <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A6" s="47">
+      <c r="A6" s="22">
         <v>46023</v>
       </c>
-      <c r="B6" s="42">
+      <c r="B6" s="17">
         <f>60</f>
         <v>60</v>
       </c>
-      <c r="C6" s="42">
+      <c r="C6" s="17">
         <v>2</v>
       </c>
-      <c r="D6" s="43">
+      <c r="D6" s="18">
         <f t="shared" si="3"/>
         <v>3.3333333333333333E-2</v>
       </c>
-      <c r="E6" s="42">
+      <c r="E6" s="17">
         <f>150</f>
         <v>150</v>
       </c>
       <c r="F6" s="11">
         <v>2.8</v>
       </c>
-      <c r="G6" s="43">
+      <c r="G6" s="18">
         <f t="shared" si="0"/>
         <v>1.8666666666666665E-2</v>
       </c>
-      <c r="H6" s="42">
+      <c r="H6" s="17">
         <f>20000</f>
         <v>20000</v>
       </c>
-      <c r="I6" s="42">
+      <c r="I6" s="17">
         <v>2456</v>
       </c>
-      <c r="J6" s="43">
+      <c r="J6" s="18">
         <f t="shared" si="1"/>
         <v>0.12280000000000001</v>
       </c>
-      <c r="K6" s="42">
+      <c r="K6" s="17">
         <f>200</f>
         <v>200</v>
       </c>
-      <c r="L6" s="42">
+      <c r="L6" s="17">
         <v>333</v>
       </c>
-      <c r="M6" s="43">
+      <c r="M6" s="18">
         <f t="shared" si="2"/>
         <v>1.665</v>
       </c>
-      <c r="N6" s="43">
+      <c r="N6" s="18">
         <f t="shared" si="4"/>
         <v>0.38357333333333332</v>
       </c>
-      <c r="O6" s="23"/>
-      <c r="P6" s="45">
+      <c r="O6" s="12"/>
+      <c r="P6" s="20">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="Q6" s="46">
+      <c r="Q6" s="21">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A7" s="47">
+      <c r="A7" s="22">
         <v>46054</v>
       </c>
-      <c r="B7" s="42">
+      <c r="B7" s="17">
         <f>60</f>
         <v>60</v>
       </c>
-      <c r="C7" s="42">
+      <c r="C7" s="17">
         <v>3</v>
       </c>
-      <c r="D7" s="43">
+      <c r="D7" s="18">
         <f t="shared" si="3"/>
         <v>0.05</v>
       </c>
-      <c r="E7" s="42">
+      <c r="E7" s="17">
         <f>150</f>
         <v>150</v>
       </c>
       <c r="F7" s="11">
         <v>9.6</v>
       </c>
-      <c r="G7" s="43">
+      <c r="G7" s="18">
         <f t="shared" si="0"/>
         <v>6.4000000000000001E-2</v>
       </c>
-      <c r="H7" s="42">
+      <c r="H7" s="17">
         <f>20000</f>
         <v>20000</v>
       </c>
-      <c r="I7" s="42">
+      <c r="I7" s="17">
         <v>2411</v>
       </c>
-      <c r="J7" s="43">
+      <c r="J7" s="18">
         <f t="shared" si="1"/>
         <v>0.12055</v>
       </c>
-      <c r="K7" s="42">
+      <c r="K7" s="17">
         <f>200</f>
         <v>200</v>
       </c>
-      <c r="L7" s="42">
+      <c r="L7" s="17">
         <v>298</v>
       </c>
-      <c r="M7" s="43">
+      <c r="M7" s="18">
         <f t="shared" si="2"/>
         <v>1.49</v>
       </c>
-      <c r="N7" s="43">
+      <c r="N7" s="18">
         <f t="shared" si="4"/>
         <v>0.36196499999999998</v>
       </c>
-      <c r="O7" s="23"/>
-      <c r="P7" s="45">
+      <c r="O7" s="12"/>
+      <c r="P7" s="20">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="Q7" s="46">
+      <c r="Q7" s="21">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
     <row r="8" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A8" s="47">
+      <c r="A8" s="22">
         <v>46082</v>
       </c>
-      <c r="B8" s="42">
+      <c r="B8" s="17">
         <f>60</f>
         <v>60</v>
       </c>
-      <c r="C8" s="42">
+      <c r="C8" s="17">
         <v>1</v>
       </c>
-      <c r="D8" s="43">
+      <c r="D8" s="18">
         <f t="shared" si="3"/>
         <v>1.6666666666666666E-2</v>
       </c>
-      <c r="E8" s="42">
+      <c r="E8" s="17">
         <f>150</f>
         <v>150</v>
       </c>
       <c r="F8" s="11">
         <v>0.12903225806451613</v>
       </c>
-      <c r="G8" s="43">
+      <c r="G8" s="18">
         <f t="shared" si="0"/>
         <v>8.6021505376344086E-4</v>
       </c>
-      <c r="H8" s="42">
+      <c r="H8" s="17">
         <f>20000</f>
         <v>20000</v>
       </c>
-      <c r="I8" s="42">
+      <c r="I8" s="17">
         <v>3336</v>
       </c>
-      <c r="J8" s="43">
+      <c r="J8" s="18">
         <f t="shared" si="1"/>
         <v>0.1668</v>
       </c>
-      <c r="K8" s="42">
+      <c r="K8" s="17">
         <f>200</f>
         <v>200</v>
       </c>
-      <c r="L8" s="42">
+      <c r="L8" s="17">
         <v>434</v>
       </c>
-      <c r="M8" s="43">
+      <c r="M8" s="18">
         <f t="shared" si="2"/>
         <v>2.17</v>
       </c>
-      <c r="N8" s="43">
+      <c r="N8" s="18">
         <f t="shared" si="4"/>
         <v>0.48921204301075272</v>
       </c>
-      <c r="O8" s="23"/>
-      <c r="P8" s="45">
+      <c r="O8" s="12"/>
+      <c r="P8" s="20">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="Q8" s="46">
+      <c r="Q8" s="21">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A9" s="47">
+      <c r="A9" s="22">
         <v>46113</v>
       </c>
-      <c r="B9" s="42">
+      <c r="B9" s="17">
         <f>60</f>
         <v>60</v>
       </c>
-      <c r="C9" s="42">
+      <c r="C9" s="17">
         <v>3</v>
       </c>
-      <c r="D9" s="43">
+      <c r="D9" s="18">
         <f t="shared" si="3"/>
         <v>0.05</v>
       </c>
-      <c r="E9" s="42">
+      <c r="E9" s="17">
         <f>150</f>
         <v>150</v>
       </c>
       <c r="F9" s="11">
         <v>1.2</v>
       </c>
-      <c r="G9" s="43">
+      <c r="G9" s="18">
         <f t="shared" si="0"/>
         <v>8.0000000000000002E-3</v>
       </c>
-      <c r="H9" s="42">
+      <c r="H9" s="17">
         <f>20000</f>
         <v>20000</v>
       </c>
-      <c r="I9" s="42">
+      <c r="I9" s="17">
         <v>2932</v>
       </c>
-      <c r="J9" s="43">
+      <c r="J9" s="18">
         <f t="shared" si="1"/>
         <v>0.14660000000000001</v>
       </c>
-      <c r="K9" s="42">
+      <c r="K9" s="17">
         <f>200</f>
         <v>200</v>
       </c>
-      <c r="L9" s="42">
+      <c r="L9" s="17">
         <v>349</v>
       </c>
-      <c r="M9" s="43">
+      <c r="M9" s="18">
         <f t="shared" si="2"/>
         <v>1.7450000000000001</v>
       </c>
-      <c r="N9" s="43">
+      <c r="N9" s="18">
         <f t="shared" si="4"/>
         <v>0.40958000000000006</v>
       </c>
-      <c r="O9" s="23"/>
-      <c r="P9" s="45">
+      <c r="O9" s="12"/>
+      <c r="P9" s="20">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="Q9" s="46">
+      <c r="Q9" s="21">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
     <row r="10" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A10" s="47">
+      <c r="A10" s="22">
         <v>46143</v>
       </c>
-      <c r="B10" s="42">
+      <c r="B10" s="17">
         <f>60</f>
         <v>60</v>
       </c>
-      <c r="C10" s="42">
+      <c r="C10" s="17">
         <v>1</v>
       </c>
-      <c r="D10" s="43">
+      <c r="D10" s="18">
         <f t="shared" si="3"/>
         <v>1.6666666666666666E-2</v>
       </c>
-      <c r="E10" s="42">
+      <c r="E10" s="17">
         <f>150</f>
         <v>150</v>
       </c>
       <c r="F10" s="11">
         <v>3.8387096774193519</v>
       </c>
-      <c r="G10" s="43">
+      <c r="G10" s="18">
         <f t="shared" si="0"/>
         <v>2.5591397849462346E-2</v>
       </c>
-      <c r="H10" s="42">
+      <c r="H10" s="17">
         <f>20000</f>
         <v>20000</v>
       </c>
-      <c r="I10" s="42">
+      <c r="I10" s="17">
         <v>4116</v>
       </c>
-      <c r="J10" s="43">
+      <c r="J10" s="18">
         <f t="shared" si="1"/>
         <v>0.20580000000000001</v>
       </c>
-      <c r="K10" s="42">
+      <c r="K10" s="17">
         <f>200</f>
         <v>200</v>
       </c>
-      <c r="L10" s="42">
+      <c r="L10" s="17">
         <v>269</v>
       </c>
-      <c r="M10" s="43">
+      <c r="M10" s="18">
         <f t="shared" si="2"/>
         <v>1.345</v>
       </c>
-      <c r="N10" s="43">
+      <c r="N10" s="18">
         <f t="shared" si="4"/>
         <v>0.34085827956989251</v>
       </c>
-      <c r="O10" s="23"/>
-      <c r="P10" s="45">
+      <c r="O10" s="12"/>
+      <c r="P10" s="20">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="Q10" s="46">
+      <c r="Q10" s="21">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="47">
+      <c r="A11" s="22">
         <v>46174</v>
       </c>
-      <c r="B11" s="42">
+      <c r="B11" s="17">
         <f>60</f>
         <v>60</v>
       </c>
-      <c r="C11" s="42">
+      <c r="C11" s="17">
         <v>3</v>
       </c>
-      <c r="D11" s="43">
+      <c r="D11" s="18">
         <f t="shared" si="3"/>
         <v>0.05</v>
       </c>
-      <c r="E11" s="42">
+      <c r="E11" s="17">
         <f>150</f>
         <v>150</v>
       </c>
       <c r="F11" s="11">
         <v>7.9333333333333176</v>
       </c>
-      <c r="G11" s="43">
+      <c r="G11" s="18">
         <f t="shared" si="0"/>
         <v>5.2888888888888784E-2</v>
       </c>
-      <c r="H11" s="42">
+      <c r="H11" s="17">
         <f>20000</f>
         <v>20000</v>
       </c>
-      <c r="I11" s="42">
+      <c r="I11" s="17">
         <v>2863</v>
       </c>
-      <c r="J11" s="43">
+      <c r="J11" s="18">
         <f t="shared" si="1"/>
         <v>0.14315</v>
       </c>
-      <c r="K11" s="42">
+      <c r="K11" s="17">
         <f>200</f>
         <v>200</v>
       </c>
-      <c r="L11" s="42">
+      <c r="L11" s="17">
         <v>259</v>
       </c>
-      <c r="M11" s="43">
+      <c r="M11" s="18">
         <f t="shared" si="2"/>
         <v>1.2949999999999999</v>
       </c>
-      <c r="N11" s="43">
+      <c r="N11" s="18">
         <f t="shared" si="4"/>
         <v>0.32752277777777777</v>
       </c>
-      <c r="O11" s="23"/>
-      <c r="P11" s="45">
+      <c r="O11" s="12"/>
+      <c r="P11" s="20">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="Q11" s="46">
+      <c r="Q11" s="21">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
     <row r="12" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A12" s="47">
+      <c r="A12" s="22">
         <v>46204</v>
       </c>
-      <c r="B12" s="42">
+      <c r="B12" s="17">
         <f>60</f>
         <v>60</v>
       </c>
-      <c r="C12" s="42">
+      <c r="C12" s="17">
         <v>2</v>
       </c>
-      <c r="D12" s="43">
+      <c r="D12" s="18">
         <f t="shared" si="3"/>
         <v>3.3333333333333333E-2</v>
       </c>
-      <c r="E12" s="42">
+      <c r="E12" s="17">
         <f>150</f>
         <v>150</v>
       </c>
       <c r="F12" s="11">
-        <v>3.2258064516129031E-2</v>
-      </c>
-      <c r="G12" s="43">
+        <v>5.7</v>
+      </c>
+      <c r="G12" s="18">
         <f t="shared" si="0"/>
-        <v>2.1505376344086021E-4</v>
-      </c>
-      <c r="H12" s="42">
+        <v>3.7999999999999999E-2</v>
+      </c>
+      <c r="H12" s="17">
         <f>20000</f>
         <v>20000</v>
       </c>
-      <c r="I12" s="42">
+      <c r="I12" s="17">
         <v>2519</v>
       </c>
-      <c r="J12" s="43">
+      <c r="J12" s="18">
         <f t="shared" si="1"/>
         <v>0.12595000000000001</v>
       </c>
-      <c r="K12" s="42">
+      <c r="K12" s="17">
         <f>200</f>
         <v>200</v>
       </c>
-      <c r="L12" s="42">
+      <c r="L12" s="17">
         <v>302</v>
       </c>
-      <c r="M12" s="43">
+      <c r="M12" s="18">
         <f t="shared" si="2"/>
         <v>1.51</v>
       </c>
-      <c r="N12" s="43">
+      <c r="N12" s="18">
         <f t="shared" si="4"/>
-        <v>0.34982801075268821</v>
-      </c>
-      <c r="O12" s="23"/>
-      <c r="P12" s="45">
+        <v>0.35738500000000006</v>
+      </c>
+      <c r="O12" s="12"/>
+      <c r="P12" s="20">
         <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="Q12" s="46">
+      <c r="Q12" s="21">
         <f t="shared" si="6"/>
         <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A13" s="47">
+      <c r="A13" s="22">
         <v>46235</v>
       </c>
-      <c r="B13" s="42"/>
-      <c r="C13" s="42"/>
-      <c r="D13" s="43">
+      <c r="B13" s="17">
+        <f>60</f>
+        <v>60</v>
+      </c>
+      <c r="C13" s="17">
+        <v>4</v>
+      </c>
+      <c r="D13" s="18">
         <f t="shared" ref="D13:D14" si="7">IFERROR(C13/B13,0)</f>
-        <v>0</v>
-      </c>
-      <c r="E13" s="42"/>
-      <c r="F13" s="11"/>
-      <c r="G13" s="43">
+        <v>6.6666666666666666E-2</v>
+      </c>
+      <c r="E13" s="17">
+        <f>150</f>
+        <v>150</v>
+      </c>
+      <c r="F13" s="11">
+        <v>27.3</v>
+      </c>
+      <c r="G13" s="18">
         <f t="shared" ref="G13:G14" si="8">IFERROR(F13/E13,0)</f>
-        <v>0</v>
-      </c>
-      <c r="H13" s="42">
+        <v>0.182</v>
+      </c>
+      <c r="H13" s="17">
         <f>20000</f>
         <v>20000</v>
       </c>
-      <c r="I13" s="42"/>
-      <c r="J13" s="43">
+      <c r="I13" s="17"/>
+      <c r="J13" s="18">
         <f t="shared" ref="J13:J14" si="9">IFERROR(I13/H13,0)</f>
         <v>0</v>
       </c>
-      <c r="K13" s="42">
+      <c r="K13" s="17">
         <f>200</f>
         <v>200</v>
       </c>
-      <c r="L13" s="42"/>
-      <c r="M13" s="43">
+      <c r="L13" s="17"/>
+      <c r="M13" s="18">
         <f t="shared" ref="M13:M14" si="10">IFERROR(L13/K13,0)</f>
         <v>0</v>
       </c>
-      <c r="N13" s="43">
+      <c r="N13" s="18">
         <f t="shared" ref="N13:N14" si="11">(D13*$B$1)+(G13*$E$1)+(J13*$H$1)+(M13*$K$1)</f>
-        <v>0</v>
-      </c>
-      <c r="O13" s="23"/>
-      <c r="P13" s="45">
+        <v>5.6400000000000006E-2</v>
+      </c>
+      <c r="O13" s="12"/>
+      <c r="P13" s="20">
         <f t="shared" ref="P13:P14" si="12">IF($O13&gt;120%,120%,IF($O13&gt;=70%,N13,IF($O13&gt;=60%,50%,0%)))</f>
         <v>0</v>
       </c>
-      <c r="Q13" s="46">
+      <c r="Q13" s="21">
         <f t="shared" ref="Q13:Q14" si="13">((F13*31)+(I13+L13))*50*P13</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A14" s="47">
+      <c r="A14" s="22">
         <v>46266</v>
       </c>
-      <c r="B14" s="42"/>
-      <c r="C14" s="42"/>
-      <c r="D14" s="43">
+      <c r="B14" s="17">
+        <f>60</f>
+        <v>60</v>
+      </c>
+      <c r="C14" s="17">
+        <v>1</v>
+      </c>
+      <c r="D14" s="18">
         <f t="shared" si="7"/>
-        <v>0</v>
-      </c>
-      <c r="E14" s="42"/>
-      <c r="F14" s="11"/>
-      <c r="G14" s="43">
+        <v>1.6666666666666666E-2</v>
+      </c>
+      <c r="E14" s="17">
+        <f>150</f>
+        <v>150</v>
+      </c>
+      <c r="F14" s="11">
+        <v>19</v>
+      </c>
+      <c r="G14" s="18">
         <f t="shared" si="8"/>
-        <v>0</v>
-      </c>
-      <c r="H14" s="42">
+        <v>0.12666666666666668</v>
+      </c>
+      <c r="H14" s="17">
         <f>20000</f>
         <v>20000</v>
       </c>
-      <c r="I14" s="42"/>
-      <c r="J14" s="43">
+      <c r="I14" s="17"/>
+      <c r="J14" s="18">
         <f t="shared" si="9"/>
         <v>0</v>
       </c>
-      <c r="K14" s="42">
+      <c r="K14" s="17">
         <f>200</f>
         <v>200</v>
       </c>
-      <c r="L14" s="42"/>
-      <c r="M14" s="43">
+      <c r="L14" s="17"/>
+      <c r="M14" s="18">
         <f t="shared" si="10"/>
         <v>0</v>
       </c>
-      <c r="N14" s="43">
+      <c r="N14" s="18">
         <f t="shared" si="11"/>
-        <v>0</v>
-      </c>
-      <c r="O14" s="23"/>
-      <c r="P14" s="45">
+        <v>3.0333333333333337E-2</v>
+      </c>
+      <c r="O14" s="12"/>
+      <c r="P14" s="20">
         <f t="shared" si="12"/>
         <v>0</v>
       </c>
-      <c r="Q14" s="46">
+      <c r="Q14" s="21">
         <f t="shared" si="13"/>
         <v>0</v>
       </c>
     </row>
+    <row r="15" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
+      <c r="A15" s="22"/>
+      <c r="B15" s="17"/>
+      <c r="C15" s="17"/>
+      <c r="D15" s="18"/>
+      <c r="E15" s="17"/>
+      <c r="F15" s="11"/>
+      <c r="G15" s="18"/>
+      <c r="H15" s="17"/>
+      <c r="I15" s="17"/>
+      <c r="J15" s="18"/>
+      <c r="K15" s="17"/>
+      <c r="L15" s="17"/>
+      <c r="M15" s="18"/>
+      <c r="N15" s="18"/>
+      <c r="P15" s="20"/>
+      <c r="Q15" s="21"/>
+    </row>
   </sheetData>
   <mergeCells count="12">
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="E1:G1"/>
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="K1:M1"/>
     <mergeCell ref="P1:P3"/>
     <mergeCell ref="Q1:Q3"/>
     <mergeCell ref="B2:D2"/>
     <mergeCell ref="E2:G2"/>
     <mergeCell ref="H2:J2"/>
     <mergeCell ref="K2:M2"/>
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="E1:G1"/>
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="K1:M1"/>
     <mergeCell ref="N1:N3"/>
   </mergeCells>
-  <conditionalFormatting sqref="G4:G14 J4:J14 M4:N14 D4:D14">
+  <conditionalFormatting sqref="D4:D15 G4:G15 J4:J15 M4:N15">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">
       <formula>0.6</formula>
     </cfRule>

</xml_diff>

<commit_message>
Remove Profil SCO Default feature completely
</commit_message>
<xml_diff>
--- a/KPI_SCO.xlsx
+++ b/KPI_SCO.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WEB REPORT\pages\sco\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{640210A1-815D-480C-A8ED-CB8CED1E1288}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD265A68-B895-4B3C-80CE-4847FA616B43}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -31552,23 +31552,27 @@
         <f>20000</f>
         <v>20000</v>
       </c>
-      <c r="I13" s="17"/>
+      <c r="I13" s="17">
+        <v>3293</v>
+      </c>
       <c r="J13" s="18">
         <f t="shared" ref="J13:J14" si="9">IFERROR(I13/H13,0)</f>
-        <v>0</v>
+        <v>0.16464999999999999</v>
       </c>
       <c r="K13" s="17">
         <f>200</f>
         <v>200</v>
       </c>
-      <c r="L13" s="17"/>
+      <c r="L13" s="17">
+        <v>200</v>
+      </c>
       <c r="M13" s="18">
         <f t="shared" ref="M13:M14" si="10">IFERROR(L13/K13,0)</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N13" s="18">
         <f t="shared" ref="N13:N14" si="11">(D13*$B$1)+(G13*$E$1)+(J13*$H$1)+(M13*$K$1)</f>
-        <v>5.6400000000000006E-2</v>
+        <v>0.30579500000000004</v>
       </c>
       <c r="O13" s="12"/>
       <c r="P13" s="20">
@@ -31610,23 +31614,27 @@
         <f>20000</f>
         <v>20000</v>
       </c>
-      <c r="I14" s="17"/>
+      <c r="I14" s="17">
+        <v>2924</v>
+      </c>
       <c r="J14" s="18">
         <f t="shared" si="9"/>
-        <v>0</v>
+        <v>0.1462</v>
       </c>
       <c r="K14" s="17">
         <f>200</f>
         <v>200</v>
       </c>
-      <c r="L14" s="17"/>
+      <c r="L14" s="17">
+        <v>344</v>
+      </c>
       <c r="M14" s="18">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1.72</v>
       </c>
       <c r="N14" s="18">
         <f t="shared" si="11"/>
-        <v>3.0333333333333337E-2</v>
+        <v>0.41819333333333336</v>
       </c>
       <c r="O14" s="12"/>
       <c r="P14" s="20">

</xml_diff>

<commit_message>
chore: update SCO performance data per cut-off 17 Okt 2026 (2026-10-20 14:41:56)
</commit_message>
<xml_diff>
--- a/KPI_SCO.xlsx
+++ b/KPI_SCO.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\WEB REPORT\pages\sco\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47DC2FDC-C10D-40EE-98FD-56AD70D615B8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB56389F-C1F3-43AA-BAAF-B8169C01C92F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="KPI_SCO" sheetId="2" r:id="rId1"/>
     <sheet name="KPI_DSO" sheetId="3" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">KPI_SCO!$A$1:$Q$52</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
 </workbook>
 </file>
@@ -482,6 +485,36 @@
     <xf numFmtId="17" fontId="11" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="10" fillId="9" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -525,36 +558,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="5" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="5" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="5" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="6" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="6" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="7" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="10" fillId="7" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -30860,69 +30863,69 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A1" s="38" t="s">
+      <c r="A1" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="B1" s="39">
+      <c r="B1" s="24">
         <v>0.3</v>
       </c>
-      <c r="C1" s="40"/>
-      <c r="D1" s="41"/>
-      <c r="E1" s="42">
+      <c r="C1" s="25"/>
+      <c r="D1" s="26"/>
+      <c r="E1" s="27">
         <v>0.2</v>
       </c>
-      <c r="F1" s="43"/>
-      <c r="G1" s="44"/>
-      <c r="H1" s="45">
+      <c r="F1" s="28"/>
+      <c r="G1" s="29"/>
+      <c r="H1" s="30">
         <v>0.3</v>
       </c>
-      <c r="I1" s="46"/>
-      <c r="J1" s="47"/>
-      <c r="K1" s="45">
+      <c r="I1" s="31"/>
+      <c r="J1" s="32"/>
+      <c r="K1" s="30">
         <v>0.2</v>
       </c>
-      <c r="L1" s="46"/>
-      <c r="M1" s="47"/>
-      <c r="N1" s="36" t="s">
+      <c r="L1" s="31"/>
+      <c r="M1" s="32"/>
+      <c r="N1" s="46" t="s">
         <v>24</v>
       </c>
       <c r="O1" s="12"/>
-      <c r="P1" s="23" t="s">
+      <c r="P1" s="33" t="s">
         <v>25</v>
       </c>
-      <c r="Q1" s="26" t="s">
+      <c r="Q1" s="36" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="2" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A2" s="38"/>
-      <c r="B2" s="27" t="s">
+      <c r="A2" s="23"/>
+      <c r="B2" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="C2" s="28"/>
-      <c r="D2" s="29"/>
-      <c r="E2" s="30" t="s">
+      <c r="C2" s="38"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="40" t="s">
         <v>28</v>
       </c>
-      <c r="F2" s="31"/>
-      <c r="G2" s="32"/>
-      <c r="H2" s="33" t="s">
+      <c r="F2" s="41"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="43" t="s">
         <v>29</v>
       </c>
-      <c r="I2" s="34"/>
-      <c r="J2" s="35"/>
-      <c r="K2" s="33" t="s">
+      <c r="I2" s="44"/>
+      <c r="J2" s="45"/>
+      <c r="K2" s="43" t="s">
         <v>30</v>
       </c>
-      <c r="L2" s="34"/>
-      <c r="M2" s="35"/>
-      <c r="N2" s="37"/>
+      <c r="L2" s="44"/>
+      <c r="M2" s="45"/>
+      <c r="N2" s="47"/>
       <c r="O2" s="12"/>
-      <c r="P2" s="24"/>
-      <c r="Q2" s="26"/>
+      <c r="P2" s="34"/>
+      <c r="Q2" s="36"/>
     </row>
     <row r="3" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
-      <c r="A3" s="38"/>
+      <c r="A3" s="23"/>
       <c r="B3" s="13" t="s">
         <v>31</v>
       </c>
@@ -30959,10 +30962,10 @@
       <c r="M3" s="15" t="s">
         <v>33</v>
       </c>
-      <c r="N3" s="37"/>
+      <c r="N3" s="47"/>
       <c r="O3" s="12"/>
-      <c r="P3" s="25"/>
-      <c r="Q3" s="26"/>
+      <c r="P3" s="35"/>
+      <c r="Q3" s="36"/>
     </row>
     <row r="4" spans="1:17" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A4" s="16">
@@ -31666,11 +31669,6 @@
     </row>
   </sheetData>
   <mergeCells count="12">
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:D1"/>
-    <mergeCell ref="E1:G1"/>
-    <mergeCell ref="H1:J1"/>
-    <mergeCell ref="K1:M1"/>
     <mergeCell ref="P1:P3"/>
     <mergeCell ref="Q1:Q3"/>
     <mergeCell ref="B2:D2"/>
@@ -31678,6 +31676,11 @@
     <mergeCell ref="H2:J2"/>
     <mergeCell ref="K2:M2"/>
     <mergeCell ref="N1:N3"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:D1"/>
+    <mergeCell ref="E1:G1"/>
+    <mergeCell ref="H1:J1"/>
+    <mergeCell ref="K1:M1"/>
   </mergeCells>
   <conditionalFormatting sqref="D4:D15 G4:G15 J4:J15 M4:N15">
     <cfRule type="cellIs" dxfId="0" priority="1" operator="lessThan">

</xml_diff>